<commit_message>
Added ngs tech slide links
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/royfr474/nbis/github/workshop-ngsintro/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08599A98-98F8-A249-9958-460F426417A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0295B050-7B25-C74D-B19B-48AB427200DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4680" yWindow="9540" windowWidth="31060" windowHeight="18920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="81">
   <si>
     <t>date</t>
   </si>
@@ -234,9 +234,6 @@
     <t>https://youtu.be/4HbSAEU5iBM</t>
   </si>
   <si>
-    <t>https://drive.google.com/file/d/15vG6VXaSL7lWNPQ6Sdn6-cxPWYHf2AAv/view?usp=sharing</t>
-  </si>
-  <si>
     <t>02/03/2026</t>
   </si>
   <si>
@@ -301,6 +298,12 @@
   </si>
   <si>
     <t>ML, AJ, PP, LA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/14kfPifL52eMTZs2jsr2ykPehFBVpAxWr/view?usp=sharing</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1U_oVEuTTKwk7zxVP_CGR5zgHP6Jd_1Oi/view?usp=sharing</t>
   </si>
 </sst>
 </file>
@@ -374,7 +377,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyProtection="1"/>
@@ -382,6 +385,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -698,10 +702,10 @@
     </row>
     <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C2" s="3">
         <v>0.375</v>
@@ -753,7 +757,7 @@
         <v>12</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>17</v>
@@ -804,7 +808,7 @@
         <v>12</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>22</v>
@@ -812,10 +816,10 @@
     </row>
     <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C8" s="3">
         <v>0.375</v>
@@ -851,7 +855,7 @@
         <v>12</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>26</v>
@@ -902,7 +906,7 @@
         <v>31</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>32</v>
@@ -948,7 +952,7 @@
         <v>12</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>38</v>
@@ -956,10 +960,10 @@
     </row>
     <row r="15" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C15" s="3">
         <v>0.375</v>
@@ -968,13 +972,13 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>57</v>
+        <v>71</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>79</v>
       </c>
       <c r="J15" s="4" t="s">
         <v>39</v>
@@ -990,10 +994,13 @@
         <v>0.5</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>71</v>
+      <c r="H16" s="7" t="s">
+        <v>80</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="5"/>
@@ -1043,7 +1050,7 @@
         <v>43</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>44</v>
@@ -1051,10 +1058,10 @@
     </row>
     <row r="20" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C20" s="3">
         <v>0.375</v>
@@ -1087,7 +1094,7 @@
         <v>43</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -1135,7 +1142,7 @@
         <v>48</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>51</v>
@@ -1143,10 +1150,10 @@
     </row>
     <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="C25" s="3">
         <v>0.375</v>
@@ -1158,7 +1165,7 @@
         <v>52</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H25" s="1" t="s">
         <v>53</v>
@@ -1177,10 +1184,10 @@
         <v>0.4375</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>55</v>
@@ -1205,7 +1212,7 @@
         <v>48</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K27" s="5"/>
     </row>
@@ -1234,7 +1241,7 @@
         <v>48</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1245,7 +1252,7 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>48</v>
@@ -1265,9 +1272,11 @@
     <hyperlink ref="J23" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="J25" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="J26" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="H15" r:id="rId13" xr:uid="{3B930BAC-E0FC-4C4D-901F-A9472A51193A}"/>
+    <hyperlink ref="H16" r:id="rId14" xr:uid="{EF0CFA49-BDC2-7C41-A9E7-23B3F5CB9036}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId13"/>
+  <legacyDrawing r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated ngs tech and pipeline slide links in schedule and contents, added note that slides and videos are not in sync
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/royfr474/nbis/github/workshop-ngsintro/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0295B050-7B25-C74D-B19B-48AB427200DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7AA20A-5EBF-6546-BD3B-1E4DFD63C737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="9540" windowWidth="31060" windowHeight="18920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2000" yWindow="10580" windowWidth="31060" windowHeight="18920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -270,9 +270,6 @@
     <t>NGS technologies</t>
   </si>
   <si>
-    <t>NGS pipelines</t>
-  </si>
-  <si>
     <t>Christian Tellgren-Roth</t>
   </si>
   <si>
@@ -304,6 +301,9 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1U_oVEuTTKwk7zxVP_CGR5zgHP6Jd_1Oi/view?usp=sharing</t>
+  </si>
+  <si>
+    <t>NGS long reads &amp; pipelines</t>
   </si>
 </sst>
 </file>
@@ -757,7 +757,7 @@
         <v>12</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>17</v>
@@ -808,7 +808,7 @@
         <v>12</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>22</v>
@@ -906,7 +906,7 @@
         <v>31</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>32</v>
@@ -975,10 +975,10 @@
         <v>68</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J15" s="4" t="s">
         <v>39</v>
@@ -994,13 +994,13 @@
         <v>0.5</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="H16" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="5"/>
@@ -1050,7 +1050,7 @@
         <v>43</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>44</v>
@@ -1094,7 +1094,7 @@
         <v>43</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -1142,7 +1142,7 @@
         <v>48</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>51</v>
@@ -1184,7 +1184,7 @@
         <v>0.4375</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>66</v>
@@ -1212,7 +1212,7 @@
         <v>48</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K27" s="5"/>
     </row>
@@ -1241,7 +1241,7 @@
         <v>48</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>